<commit_message>
Daily EOD data and reports for 2026-09-30
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260930.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260930.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.895</v>
+        <v>1.865</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.015</v>
+        <v>-0.015</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.80%</t>
+          <t>-0.80%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>290277.99</v>
+        <v>285682.57</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2297.72</v>
+        <v>-2297.71</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.555</v>
+        <v>2.6</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.025</v>
+        <v>0.02</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.97%</t>
+          <t>0.78%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>178850</v>
+        <v>182000</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-1750</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>60.94</v>
+        <v>60.82</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.31</v>
+        <v>0.19</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.51%</t>
+          <t>0.31%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>487520</v>
+        <v>486560</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>2480</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.004</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0</v>
+        <v>176.36</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-176.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>149.22</v>
+        <v>151.01</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-1.05</v>
+        <v>0.74</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.70%</t>
+          <t>0.49%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.025</v>
+        <v>0.035</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.82%</t>
+          <t>3.95%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>9100</v>
+        <v>9200</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>250</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>182</v>
+        <v>184.22</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.3</v>
+        <v>1.92</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>1.05%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>728000</v>
+        <v>736880</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-1200</v>
+        <v>7680</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.235</v>
+        <v>0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>2.13%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4700</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>15.5</v>
+        <v>15.52</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0.13%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>47197.5</v>
+        <v>47258.4</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.089</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.08500000000000001</v>
+        <v>0.004</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>4.71%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>837.67</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-800.02</v>
+        <v>37.65</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.089</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.089</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>534</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.76</v>
+        <v>35.07</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.26</v>
+        <v>0.05</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>0.14%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>31.52</v>
+        <v>31.88</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.04</v>
+        <v>0.4</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.13%</t>
+          <t>1.27%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>40597.76</v>
+        <v>41061.44</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>51.52</v>
+        <v>515.2</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1781543.26</v>
+        <v>1794990.43</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-5481.15</v>
+        <v>7966.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>